<commit_message>
Back with some small updates
</commit_message>
<xml_diff>
--- a/excel/legends_info.xlsx
+++ b/excel/legends_info.xlsx
@@ -243,7 +243,7 @@
     <t>1900-8-26</t>
   </si>
   <si>
-    <t>Loading biography…..</t>
+    <t>The final piece of the legendary Dragon Ball squad to start the dynasty and become one of the top teams not only in the AFC Manga League but also in the international tournaments. Although he had a rough start from the beginning, he still make the spot to be one of the best keepers in the world by crucial saves and an impressive ability to understand and analyze the situation to help the team making their plans for the next movements. Every player had faced against him knows how dangerous he was when he was on the pitch, and considered him as the “Silent Hero” of the team.</t>
   </si>
 </sst>
 </file>
@@ -354,7 +354,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -374,6 +374,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1549,7 +1552,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" ht="20.05" customHeight="1">
+    <row r="6" ht="176" customHeight="1">
       <c r="A6" t="s" s="5">
         <v>26</v>
       </c>
@@ -1568,153 +1571,153 @@
       <c r="F6" s="6">
         <v>178</v>
       </c>
-      <c r="G6" t="s" s="5">
+      <c r="G6" t="s" s="7">
         <v>29</v>
       </c>
     </row>
     <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
     </row>
     <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
     </row>
     <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
     </row>
     <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
     </row>
     <row r="11" ht="20.05" customHeight="1">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
     </row>
     <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
     </row>
     <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
     </row>
     <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
     </row>
     <row r="15" ht="20.05" customHeight="1">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
     </row>
     <row r="16" ht="20.05" customHeight="1">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
     </row>
     <row r="17" ht="20.05" customHeight="1">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
     </row>
     <row r="18" ht="20.05" customHeight="1">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
     </row>
     <row r="19" ht="20.05" customHeight="1">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
     </row>
     <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
     </row>
     <row r="21" ht="20.05" customHeight="1">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
     </row>
     <row r="22" ht="20.05" customHeight="1">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>